<commit_message>
docs: report entry for the 0008 date fix
</commit_message>
<xml_diff>
--- a/Reports/Registration-Setup-Test-Report.xlsx
+++ b/Reports/Registration-Setup-Test-Report.xlsx
@@ -11825,7 +11825,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>db-migrations.int.spec.ts: suspensions carried over, published ones back to draft. Also applied by hand on kando-dev (0 rows changed).</t>
+          <t>db-migrations.int.spec.ts: suspensions carried over, published ones back to draft. Also applied by hand on kando-dev (0 rows changed). Legacy rows are read through the domain mappers.</t>
         </is>
       </c>
     </row>
@@ -11862,7 +11862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -12652,6 +12652,23 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Fixed (re-review, Important): 0008 suspension without a date</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>The legacy flag now becomes 9999-12-31, not infinity (Node read infinity as Invalid Date and the profile and admin provider reads threw). The migration test reads legacy rows through getMyProfile and adminGet and checks they stay hidden (f7eb8ce). Dev database unaffected: no such row.</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: report and README: the two tab tests, 390 tests in total
</commit_message>
<xml_diff>
--- a/Reports/Registration-Setup-Test-Report.xlsx
+++ b/Reports/Registration-Setup-Test-Report.xlsx
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Test Results'!C2:C389)</f>
+        <f>COUNTA('Test Results'!C2:C391)</f>
         <v/>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E389"/>
+  <dimension ref="A1:E391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11078,6 +11078,60 @@
         </is>
       </c>
       <c r="E389" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="4" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B390" s="4" t="inlineStr">
+        <is>
+          <t>profile-tab.test.ts</t>
+        </is>
+      </c>
+      <c r="C390" s="4" t="inlineStr">
+        <is>
+          <t>the My profile tab shows only for a known provider</t>
+        </is>
+      </c>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="E390" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="4" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B391" s="4" t="inlineStr">
+        <is>
+          <t>profile-tab.test.ts</t>
+        </is>
+      </c>
+      <c r="C391" s="4" t="inlineStr">
+        <is>
+          <t>after sign-out the next account does not inherit the provider tab</t>
+        </is>
+      </c>
+      <c r="D391" s="4" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="E391" s="4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -11253,7 +11307,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>108 tests.</t>
+          <t>110 tests.</t>
         </is>
       </c>
     </row>
@@ -11862,7 +11916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -12669,6 +12723,23 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>My profile tab only for providers (PR #9)</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Owner decision: customers reach the profile page through Account &gt; Offer services; the tab appears once they are providers. Two jest tests added (110 app tests). Phone check: customer sees no tab; Offer services opens the page; tab appears after the draft exists.</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Not yet done (phone)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(app): My profile tab only for providers (carries PR #9 into main) (#10)
* feat(app): My profile tab only for providers; customers use Account > Offer services

* docs: report and README: the two tab tests, 390 tests in total
</commit_message>
<xml_diff>
--- a/Reports/Registration-Setup-Test-Report.xlsx
+++ b/Reports/Registration-Setup-Test-Report.xlsx
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Test Results'!C2:C389)</f>
+        <f>COUNTA('Test Results'!C2:C391)</f>
         <v/>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E389"/>
+  <dimension ref="A1:E391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11078,6 +11078,60 @@
         </is>
       </c>
       <c r="E389" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="4" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B390" s="4" t="inlineStr">
+        <is>
+          <t>profile-tab.test.ts</t>
+        </is>
+      </c>
+      <c r="C390" s="4" t="inlineStr">
+        <is>
+          <t>the My profile tab shows only for a known provider</t>
+        </is>
+      </c>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="E390" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="4" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B391" s="4" t="inlineStr">
+        <is>
+          <t>profile-tab.test.ts</t>
+        </is>
+      </c>
+      <c r="C391" s="4" t="inlineStr">
+        <is>
+          <t>after sign-out the next account does not inherit the provider tab</t>
+        </is>
+      </c>
+      <c r="D391" s="4" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="E391" s="4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -11253,7 +11307,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>108 tests.</t>
+          <t>110 tests.</t>
         </is>
       </c>
     </row>
@@ -11862,7 +11916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -12669,6 +12723,23 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>My profile tab only for providers (PR #9)</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Owner decision: customers reach the profile page through Account &gt; Offer services; the tab appears once they are providers. Two jest tests added (110 app tests). Phone check: customer sees no tab; Offer services opens the page; tab appears after the draft exists.</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Not yet done (phone)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: report and README counts after the navigation hand-off
</commit_message>
<xml_diff>
--- a/Reports/Registration-Setup-Test-Report.xlsx
+++ b/Reports/Registration-Setup-Test-Report.xlsx
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Test Results'!C2:C398)</f>
+        <f>COUNTA('Test Results'!C2:C402)</f>
         <v/>
       </c>
     </row>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Results'!E2:E398,"Passed")</f>
+        <f>COUNTIF('Test Results'!E2:E402,"Passed")</f>
         <v/>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Results'!E2:E398,"Failed")</f>
+        <f>COUNTIF('Test Results'!E2:E402,"Failed")</f>
         <v/>
       </c>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Test Results'!E2:E398,"Skipped")</f>
+        <f>COUNTIF('Test Results'!E2:E402,"Skipped")</f>
         <v/>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7603,17 +7603,17 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>index.test.ts</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
-          <t>creates the draft, reloads /me, then opens the profile page, in that order</t>
+          <t>texts come from the shared catalogue, in the chosen language, with placeholders filled</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr">
@@ -7630,17 +7630,17 @@
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>index.test.ts</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr">
         <is>
-          <t>welcome passes through to the page</t>
+          <t>the translate button texts exist in both languages</t>
         </is>
       </c>
       <c r="D262" s="4" t="inlineStr">
@@ -7657,17 +7657,17 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>index.test.ts</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>a failure returns the error text and does not navigate</t>
+          <t>errorText maps the auth server codes to catalogue messages</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
@@ -7684,17 +7684,17 @@
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>index.test.ts</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
-          <t>a second call while one runs does nothing extra</t>
+          <t>errorText maps the app API strings</t>
         </is>
       </c>
       <c r="D264" s="4" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>texts come from the shared catalogue, in the chosen language, with placeholders filled</t>
+          <t>docText maps known document codes and passes unknown ones through</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
@@ -7738,17 +7738,17 @@
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Share profile</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>share-profile.test.ts</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>the translate button texts exist in both languages</t>
+          <t>the provider page url carries the language only when it is not the default</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
@@ -7765,17 +7765,17 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Share profile</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>share-profile.test.ts</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>errorText maps the auth server codes to catalogue messages</t>
+          <t>shareProfile passes the url and the text in the given language</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
@@ -7792,17 +7792,17 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>errorText maps the app API strings</t>
+          <t>creates the draft, reloads /me, then sets the target, in that order</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
@@ -7819,17 +7819,17 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>docText maps known document codes and passes unknown ones through</t>
+          <t>welcome passes through</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
@@ -7846,17 +7846,17 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>Share profile</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>share-profile.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>the provider page url carries the language only when it is not the default</t>
+          <t>a failure returns the error text and does not navigate</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
@@ -7873,17 +7873,17 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>Share profile</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>share-profile.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>shareProfile passes the url and the text in the given language</t>
+          <t>a second call while one runs does nothing extra</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
@@ -8278,17 +8278,17 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>preparePhoto keeps the long side at 1600 px</t>
+          <t>set, consume once, then nothing</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
@@ -8305,17 +8305,17 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>tooLarge is true above 4_434_464 bytes</t>
+          <t>clearPending drops it (sign-out)</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
@@ -8332,17 +8332,17 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>pickPhoto cancelled is null</t>
+          <t>readyToNavigate: only with a target and a visible profile tab</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
@@ -8364,12 +8364,12 @@
       </c>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>pickPhoto a refused permission is denied, not cancelled</t>
+          <t>server errors land on the right field</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
@@ -8391,12 +8391,12 @@
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>pickDocument offers PDFs and the image types the server accepts, from any file source</t>
+          <t>withItem adds a trimmed new skill or strength once and ignores blanks</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
@@ -8418,12 +8418,12 @@
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>pickDocument cancelled is null</t>
+          <t>the form-level error shows unless every server error has an inline slot</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>server errors land on the right field</t>
+          <t>service and reference validation</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
@@ -8477,7 +8477,7 @@
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>withItem adds a trimmed new skill or strength once and ignores blanks</t>
+          <t>every missing item the publish route can return has de and en text</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>the form-level error shows unless every server error has an inline slot</t>
+          <t>the service body names the category by id and the currency, as the server expects</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>service and reference validation</t>
+          <t>a 400 "Invalid input" marks each named field</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>every missing item the publish route can return has de and en text</t>
+          <t>live means published and not suspended now (the server rule of listServices)</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
@@ -8580,12 +8580,12 @@
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>the service body names the category by id and the currency, as the server expects</t>
+          <t>preparePhoto keeps the long side at 1600 px</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
@@ -8607,12 +8607,12 @@
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>a 400 "Invalid input" marks each named field</t>
+          <t>tooLarge is true above 4_434_464 bytes</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
@@ -8634,12 +8634,12 @@
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>live means published and not suspended now (the server rule of listServices)</t>
+          <t>pickPhoto cancelled is null</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
@@ -8661,12 +8661,12 @@
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>sends the stored cookie and stores a new set-cookie</t>
+          <t>pickPhoto a refused permission is denied, not cancelled</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
@@ -8688,12 +8688,12 @@
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>a single joined set-cookie header (no getSetCookie) is split into its cookies</t>
+          <t>pickDocument offers PDFs and the image types the server accepts, from any file source</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
@@ -8715,12 +8715,12 @@
       </c>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>clears the session on 401</t>
+          <t>pickDocument cancelled is null</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
@@ -8742,12 +8742,12 @@
       </c>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>a 401 without a stored session does not call onUnauthorized</t>
+          <t>no rows when no service needs a document</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
@@ -8769,12 +8769,12 @@
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>every request names the app origin and leaves the platform cookie store out</t>
+          <t>a babysitting service with nothing uploaded â†’ police-certificate none</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
@@ -8796,12 +8796,12 @@
       </c>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>a 409 with error and missing throws ApiError with code and missing</t>
+          <t>the most recently reviewed check decides, like the server</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
@@ -8823,12 +8823,12 @@
       </c>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>a 400 "Invalid input" lists the fields named by its issues</t>
+          <t>a pending check shows pending even after an approval</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
@@ -8850,12 +8850,12 @@
       </c>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>a network failure throws ApiError(0, network)</t>
+          <t>a requirement code the app does not know still gets a row, after the known ones</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
@@ -8877,12 +8877,12 @@
       </c>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>a server that never answers fails as network after the time limit</t>
+          <t>two services needing the same document give one row</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
@@ -8904,12 +8904,12 @@
       </c>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>saves have no time limit: a slow save that succeeds is not reported as a failure</t>
+          <t>two different categories needing the same document give one row with the latest status</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
@@ -8931,12 +8931,12 @@
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>updateMe PATCHes the account name</t>
+          <t>a hidden service says a document is needed until it is uploaded, then that it waits for the check</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
@@ -8958,12 +8958,12 @@
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>upload sends multipart with the cookie and no time limit</t>
+          <t>sharing is allowed only while no service waits for a document</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
@@ -8985,12 +8985,12 @@
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>upload sends the file bytes with its name and type, not a bare { uri } object</t>
+          <t>saving a waiting service keeps Share hidden: the server answer carries waitingFor</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
@@ -9007,17 +9007,17 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use flash</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>use-flash.test.ts</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>a file the phone cannot open is "File unreadable", not a network error, and nothing is sent</t>
+          <t>createFlash: on after show, off after the delay, off at once on hide, a second show restarts the delay</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
@@ -9034,17 +9034,17 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use flash</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>use-flash.test.ts</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>upload maps a 413 to ApiError "File too large"</t>
+          <t>createFlash: show is a no-op after dispose</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
@@ -9066,12 +9066,12 @@
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>upload maps a network failure to ApiError network and does not retry</t>
+          <t>prices follow the website rules in German and English</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
@@ -9093,12 +9093,12 @@
       </c>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>a store that cannot be read (Keystore failure) sends the request without a cookie</t>
+          <t>distance shows km, remote or nothing</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
@@ -9120,12 +9120,12 @@
       </c>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>a cookie that cannot be saved does not fail a request the server already carried out</t>
+          <t>search path leaves out empty filters and trims text</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
@@ -9147,12 +9147,12 @@
       </c>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>a malformed Set-Cookie line without "=" is skipped</t>
+          <t>photoSrc loads only absolute http(s) URLs, never a server-relative /api path</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
@@ -9174,12 +9174,12 @@
       </c>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>translation.test.ts</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>updateMe sends the one-field name as first and last name, split at the last space</t>
+          <t>applyTexts swaps only the translatable fields and keeps names, prices and photos</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
@@ -9201,12 +9201,12 @@
       </c>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>translation.test.ts</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>prices follow the website rules in German and English</t>
+          <t>applyTexts matches services and references by id and leaves unknown ones untouched</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
@@ -9228,12 +9228,12 @@
       </c>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>translation.test.ts</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>distance shows km, remote or nothing</t>
+          <t>applyTexts keeps line breaks</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
@@ -9255,12 +9255,12 @@
       </c>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>search path leaves out empty filters and trims text</t>
+          <t>sends the stored cookie and stores a new set-cookie</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
@@ -9282,12 +9282,12 @@
       </c>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>photoSrc loads only absolute http(s) URLs, never a server-relative /api path</t>
+          <t>a single joined set-cookie header (no getSetCookie) is split into its cookies</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
@@ -9309,12 +9309,12 @@
       </c>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>my-profile.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>a failed check after the upload deletes the uploaded file and reports the original error</t>
+          <t>clears the session on 401</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
@@ -9336,12 +9336,12 @@
       </c>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>my-profile.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>a successful submit deletes nothing</t>
+          <t>a 401 without a stored session does not call onUnauthorized</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
@@ -9363,12 +9363,12 @@
       </c>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>my-profile.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>a failing clean-up does not hide the original error</t>
+          <t>every request names the app origin and leaves the platform cookie store out</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
@@ -9390,12 +9390,12 @@
       </c>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>auth-layout.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>logged-out landing route is login</t>
+          <t>a 409 with error and missing throws ApiError with code and missing</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
@@ -9417,12 +9417,12 @@
       </c>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>auth-layout.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>no test files inside src/app (each file there becomes a screen)</t>
+          <t>a 400 "Invalid input" lists the fields named by its issues</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
@@ -9439,17 +9439,17 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>Serial create</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>serial-create.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>choosing twice before the create returns creates once, then updates</t>
+          <t>a network failure throws ApiError(0, network)</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
@@ -9466,17 +9466,17 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>Serial create</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>serial-create.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>an existing id is only updated</t>
+          <t>a server that never answers fails as network after the time limit</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
@@ -9493,17 +9493,17 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>two quick changes become one request with the last value</t>
+          <t>saves have no time limit: a slow save that succeeds is not reported as a failure</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
@@ -9520,17 +9520,17 @@
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>flush saves immediately and nothing is sent twice</t>
+          <t>updateMe PATCHes the account name</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
@@ -9547,17 +9547,17 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>a rejected save marks error and retry resends the same value</t>
+          <t>upload sends multipart with the cookie and no time limit</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
@@ -9574,17 +9574,17 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>a change typed while a save is in flight is sent after it, in order</t>
+          <t>upload sends the file bytes with its name and type, not a bare { uri } object</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
@@ -9601,17 +9601,17 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>dispose sends a pending change so nothing typed is lost</t>
+          <t>a file the phone cannot open is "File unreadable", not a network error, and nothing is sent</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
@@ -9633,12 +9633,12 @@
       </c>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>loading -&gt; signed in -&gt; signed out</t>
+          <t>upload maps a 413 to ApiError "File too large"</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
@@ -9660,12 +9660,12 @@
       </c>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>an unverified email never counts as signed in: sign-in sends a code and asks for it</t>
+          <t>upload maps a network failure to ApiError network and does not retry</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
@@ -9687,12 +9687,12 @@
       </c>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>a server that refuses unverified sign-ins (EMAIL_NOT_VERIFIED) also leads to the code screen</t>
+          <t>a store that cannot be read (Keystore failure) sends the request without a cookie</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
@@ -9714,12 +9714,12 @@
       </c>
       <c r="B339" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C339" s="4" t="inlineStr">
         <is>
-          <t>sign-up creates the account and sends the code; the right code signs in and saves the account name</t>
+          <t>a cookie that cannot be saved does not fail a request the server already carried out</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
@@ -9741,12 +9741,12 @@
       </c>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>a wrong code throws and keeps signed out</t>
+          <t>a malformed Set-Cookie line without "=" is skipped</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
@@ -9768,12 +9768,12 @@
       </c>
       <c r="B341" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>a failed login rejects and keeps signed out; a server error on load means signed out</t>
+          <t>updateMe sends the one-field name as first and last name, split at the last space</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -9795,12 +9795,12 @@
       </c>
       <c r="B342" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>my-profile.test.ts</t>
         </is>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>a network error on load sets offline (not signed out); retry recovers</t>
+          <t>a failed check after the upload deletes the uploaded file and reports the original error</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
@@ -9822,12 +9822,12 @@
       </c>
       <c r="B343" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>my-profile.test.ts</t>
         </is>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>onUnauthorized from the API client signs the user out</t>
+          <t>a successful submit deletes nothing</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
@@ -9849,12 +9849,12 @@
       </c>
       <c r="B344" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>my-profile.test.ts</t>
         </is>
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
-          <t>switching the language also saves it for emails, but only while signed in</t>
+          <t>a failing clean-up does not hide the original error</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
@@ -9871,17 +9871,17 @@
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B345" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t>verify finishes the sign-up: names and address, then the picture, then the record is cleared; returns the tick</t>
+          <t>two quick changes become one request with the last value</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
@@ -9898,17 +9898,17 @@
     <row r="346">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B346" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
-          <t>a failed upload keeps the record; loadSession retries it once and clears it</t>
+          <t>flush saves immediately and nothing is sent twice</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
@@ -9925,17 +9925,17 @@
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B347" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
-          <t>loadSession without a record or while signed out does not finish a sign-up</t>
+          <t>a rejected save marks error and retry resends the same value</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
@@ -9952,17 +9952,17 @@
     <row r="348">
       <c r="A348" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B348" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C348" s="4" t="inlineStr">
         <is>
-          <t>a record for another email is dropped and applies nothing</t>
+          <t>a change typed while a save is in flight is sent after it, in order</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
@@ -9979,17 +9979,17 @@
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B349" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C349" s="4" t="inlineStr">
         <is>
-          <t>a failed PATCH keeps the full record</t>
+          <t>dispose sends a pending change so nothing typed is lost</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
@@ -10006,17 +10006,17 @@
     <row r="350">
       <c r="A350" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Stale guard</t>
         </is>
       </c>
       <c r="B350" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>stale-guard.test.ts</t>
         </is>
       </c>
       <c r="C350" s="4" t="inlineStr">
         <is>
-          <t>after the PATCH succeeded, a failed upload keeps only email, tick and picture; the retry does not PATCH again</t>
+          <t>a response older than one already applied is ignored</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr">
@@ -10033,17 +10033,17 @@
     <row r="351">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Stale guard</t>
         </is>
       </c>
       <c r="B351" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>stale-guard.test.ts</t>
         </is>
       </c>
       <c r="C351" s="4" t="inlineStr">
         <is>
-          <t>a picture whose cached file is gone is dropped and the record cleared</t>
+          <t>answers arriving in order are all applied</t>
         </is>
       </c>
       <c r="D351" s="4" t="inlineStr">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="C352" s="4" t="inlineStr">
         <is>
-          <t>sign-up keeps the record for the code step; a failed sign-up leaves none</t>
+          <t>loading -&gt; signed in -&gt; signed out</t>
         </is>
       </c>
       <c r="D352" s="4" t="inlineStr">
@@ -10097,7 +10097,7 @@
       </c>
       <c r="C353" s="4" t="inlineStr">
         <is>
-          <t>finishing a sign-up reloads /me so the home nudge sees the new picture; nothing to finish, nothing to reload</t>
+          <t>an unverified email never counts as signed in: sign-in sends a code and asks for it</t>
         </is>
       </c>
       <c r="D353" s="4" t="inlineStr">
@@ -10114,17 +10114,17 @@
     <row r="354">
       <c r="A354" s="4" t="inlineStr">
         <is>
-          <t>Use flash</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B354" s="4" t="inlineStr">
         <is>
-          <t>use-flash.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C354" s="4" t="inlineStr">
         <is>
-          <t>createFlash: on after show, off after the delay, off at once on hide, a second show restarts the delay</t>
+          <t>a server that refuses unverified sign-ins (EMAIL_NOT_VERIFIED) also leads to the code screen</t>
         </is>
       </c>
       <c r="D354" s="4" t="inlineStr">
@@ -10146,12 +10146,12 @@
       </c>
       <c r="B355" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>no rows when no service needs a document</t>
+          <t>sign-up creates the account and sends the code; the right code signs in and saves the account name</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr">
@@ -10173,12 +10173,12 @@
       </c>
       <c r="B356" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C356" s="4" t="inlineStr">
         <is>
-          <t>a babysitting service with nothing uploaded â†’ police-certificate none</t>
+          <t>a wrong code throws and keeps signed out</t>
         </is>
       </c>
       <c r="D356" s="4" t="inlineStr">
@@ -10200,12 +10200,12 @@
       </c>
       <c r="B357" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C357" s="4" t="inlineStr">
         <is>
-          <t>the most recently reviewed check decides, like the server</t>
+          <t>a failed login rejects and keeps signed out; a server error on load means signed out</t>
         </is>
       </c>
       <c r="D357" s="4" t="inlineStr">
@@ -10227,12 +10227,12 @@
       </c>
       <c r="B358" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C358" s="4" t="inlineStr">
         <is>
-          <t>a pending check shows pending even after an approval</t>
+          <t>a network error on load sets offline (not signed out); retry recovers</t>
         </is>
       </c>
       <c r="D358" s="4" t="inlineStr">
@@ -10254,12 +10254,12 @@
       </c>
       <c r="B359" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
-          <t>a requirement code the app does not know still gets a row, after the known ones</t>
+          <t>onUnauthorized from the API client signs the user out</t>
         </is>
       </c>
       <c r="D359" s="4" t="inlineStr">
@@ -10281,12 +10281,12 @@
       </c>
       <c r="B360" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C360" s="4" t="inlineStr">
         <is>
-          <t>two services needing the same document give one row</t>
+          <t>switching the language also saves it for emails, but only while signed in</t>
         </is>
       </c>
       <c r="D360" s="4" t="inlineStr">
@@ -10308,12 +10308,12 @@
       </c>
       <c r="B361" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C361" s="4" t="inlineStr">
         <is>
-          <t>two different categories needing the same document give one row with the latest status</t>
+          <t>verify finishes the sign-up: names and address, then the picture, then the record is cleared; returns the tick</t>
         </is>
       </c>
       <c r="D361" s="4" t="inlineStr">
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B362" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C362" s="4" t="inlineStr">
         <is>
-          <t>a hidden service says a document is needed until it is uploaded, then that it waits for the check</t>
+          <t>a failed upload keeps the record; loadSession retries it once and clears it</t>
         </is>
       </c>
       <c r="D362" s="4" t="inlineStr">
@@ -10362,12 +10362,12 @@
       </c>
       <c r="B363" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C363" s="4" t="inlineStr">
         <is>
-          <t>sharing is allowed only while no service waits for a document</t>
+          <t>loadSession without a record or while signed out does not finish a sign-up</t>
         </is>
       </c>
       <c r="D363" s="4" t="inlineStr">
@@ -10389,12 +10389,12 @@
       </c>
       <c r="B364" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C364" s="4" t="inlineStr">
         <is>
-          <t>saving a waiting service keeps Share hidden: the server answer carries waitingFor</t>
+          <t>a record for another email is dropped and applies nothing</t>
         </is>
       </c>
       <c r="D364" s="4" t="inlineStr">
@@ -10411,17 +10411,17 @@
     <row r="365">
       <c r="A365" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B365" s="4" t="inlineStr">
         <is>
-          <t>profile-tab.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C365" s="4" t="inlineStr">
         <is>
-          <t>the My profile tab shows only for a known provider</t>
+          <t>a failed PATCH keeps the full record</t>
         </is>
       </c>
       <c r="D365" s="4" t="inlineStr">
@@ -10438,17 +10438,17 @@
     <row r="366">
       <c r="A366" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B366" s="4" t="inlineStr">
         <is>
-          <t>profile-tab.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C366" s="4" t="inlineStr">
         <is>
-          <t>after sign-out the next account does not inherit the provider tab</t>
+          <t>after the PATCH succeeded, a failed upload keeps only email, tick and picture; the retry does not PATCH again</t>
         </is>
       </c>
       <c r="D366" s="4" t="inlineStr">
@@ -10465,17 +10465,17 @@
     <row r="367">
       <c r="A367" s="4" t="inlineStr">
         <is>
-          <t>Picture nudge</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B367" s="4" t="inlineStr">
         <is>
-          <t>picture-nudge.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C367" s="4" t="inlineStr">
         <is>
-          <t>the dismissed-nudge key is per user, so a second account on the device still sees it</t>
+          <t>a picture whose cached file is gone is dropped and the record cleared</t>
         </is>
       </c>
       <c r="D367" s="4" t="inlineStr">
@@ -10497,12 +10497,12 @@
       </c>
       <c r="B368" s="4" t="inlineStr">
         <is>
-          <t>translation.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C368" s="4" t="inlineStr">
         <is>
-          <t>applyTexts swaps only the translatable fields and keeps names, prices and photos</t>
+          <t>sign-up keeps the record for the code step; a failed sign-up leaves none</t>
         </is>
       </c>
       <c r="D368" s="4" t="inlineStr">
@@ -10524,12 +10524,12 @@
       </c>
       <c r="B369" s="4" t="inlineStr">
         <is>
-          <t>translation.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C369" s="4" t="inlineStr">
         <is>
-          <t>applyTexts matches services and references by id and leaves unknown ones untouched</t>
+          <t>finishing a sign-up reloads /me so the home nudge sees the new picture; nothing to finish, nothing to reload</t>
         </is>
       </c>
       <c r="D369" s="4" t="inlineStr">
@@ -10546,17 +10546,17 @@
     <row r="370">
       <c r="A370" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Pending signup</t>
         </is>
       </c>
       <c r="B370" s="4" t="inlineStr">
         <is>
-          <t>translation.test.ts</t>
+          <t>pending-signup.test.ts</t>
         </is>
       </c>
       <c r="C370" s="4" t="inlineStr">
         <is>
-          <t>applyTexts keeps line breaks</t>
+          <t>the pending record round-trips and clears</t>
         </is>
       </c>
       <c r="D370" s="4" t="inlineStr">
@@ -10573,17 +10573,17 @@
     <row r="371">
       <c r="A371" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Picture nudge</t>
         </is>
       </c>
       <c r="B371" s="4" t="inlineStr">
         <is>
-          <t>match.test.ts</t>
+          <t>picture-nudge.test.ts</t>
         </is>
       </c>
       <c r="C371" s="4" t="inlineStr">
         <is>
-          <t>matches ignores case and accents, and an empty query matches everything</t>
+          <t>the dismissed-nudge key is per user, so a second account on the device still sees it</t>
         </is>
       </c>
       <c r="D371" s="4" t="inlineStr">
@@ -10600,17 +10600,17 @@
     <row r="372">
       <c r="A372" s="4" t="inlineStr">
         <is>
-          <t>Pending signup</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B372" s="4" t="inlineStr">
         <is>
-          <t>pending-signup.test.ts</t>
+          <t>match.test.ts</t>
         </is>
       </c>
       <c r="C372" s="4" t="inlineStr">
         <is>
-          <t>the pending record round-trips and clears</t>
+          <t>matches ignores case and accents, and an empty query matches everything</t>
         </is>
       </c>
       <c r="D372" s="4" t="inlineStr">
@@ -10627,17 +10627,17 @@
     <row r="373">
       <c r="A373" s="4" t="inlineStr">
         <is>
-          <t>Use me</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B373" s="4" t="inlineStr">
         <is>
-          <t>use-me.test.ts</t>
+          <t>profile-tab.test.ts</t>
         </is>
       </c>
       <c r="C373" s="4" t="inlineStr">
         <is>
-          <t>a loadMe in flight at sign-out never fills the store for the next account</t>
+          <t>the My profile tab shows only for a known provider</t>
         </is>
       </c>
       <c r="D373" s="4" t="inlineStr">
@@ -10654,17 +10654,17 @@
     <row r="374">
       <c r="A374" s="4" t="inlineStr">
         <is>
-          <t>Stale guard</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B374" s="4" t="inlineStr">
         <is>
-          <t>stale-guard.test.ts</t>
+          <t>profile-tab.test.ts</t>
         </is>
       </c>
       <c r="C374" s="4" t="inlineStr">
         <is>
-          <t>a response older than one already applied is ignored</t>
+          <t>after sign-out the next account does not inherit the provider tab</t>
         </is>
       </c>
       <c r="D374" s="4" t="inlineStr">
@@ -10681,17 +10681,17 @@
     <row r="375">
       <c r="A375" s="4" t="inlineStr">
         <is>
-          <t>Stale guard</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B375" s="4" t="inlineStr">
         <is>
-          <t>stale-guard.test.ts</t>
+          <t>auth-layout.test.ts</t>
         </is>
       </c>
       <c r="C375" s="4" t="inlineStr">
         <is>
-          <t>answers arriving in order are all applied</t>
+          <t>logged-out landing route is login</t>
         </is>
       </c>
       <c r="D375" s="4" t="inlineStr">
@@ -10708,22 +10708,22 @@
     <row r="376">
       <c r="A376" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B376" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>auth-layout.test.ts</t>
         </is>
       </c>
       <c r="C376" s="4" t="inlineStr">
         <is>
-          <t>ServiceInputSchema rejects three decimals and negative prices</t>
+          <t>no test files inside src/app (each file there becomes a screen)</t>
         </is>
       </c>
       <c r="D376" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E376" s="4" t="inlineStr">
@@ -10735,22 +10735,22 @@
     <row r="377">
       <c r="A377" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Serial create</t>
         </is>
       </c>
       <c r="B377" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>serial-create.test.ts</t>
         </is>
       </c>
       <c r="C377" s="4" t="inlineStr">
         <is>
-          <t>ServiceInputSchema needs no price on request</t>
+          <t>choosing twice before the create returns creates once, then updates</t>
         </is>
       </c>
       <c r="D377" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E377" s="4" t="inlineStr">
@@ -10762,22 +10762,22 @@
     <row r="378">
       <c r="A378" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Serial create</t>
         </is>
       </c>
       <c r="B378" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>serial-create.test.ts</t>
         </is>
       </c>
       <c r="C378" s="4" t="inlineStr">
         <is>
-          <t>AdminListQuerySchema caps pageSize at 100</t>
+          <t>an existing id is only updated</t>
         </is>
       </c>
       <c r="D378" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E378" s="4" t="inlineStr">
@@ -10789,22 +10789,22 @@
     <row r="379">
       <c r="A379" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Use me</t>
         </is>
       </c>
       <c r="B379" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>use-me.test.ts</t>
         </is>
       </c>
       <c r="C379" s="4" t="inlineStr">
         <is>
-          <t>parse helpers parseBody answers 400 with the issues</t>
+          <t>a loadMe in flight at sign-out never fills the store for the next account</t>
         </is>
       </c>
       <c r="D379" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E379" s="4" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="C380" s="4" t="inlineStr">
         <is>
-          <t>parse helpers parseQuery reads the search params</t>
+          <t>ServiceInputSchema rejects three decimals and negative prices</t>
         </is>
       </c>
       <c r="D380" s="4" t="inlineStr">
@@ -10853,7 +10853,7 @@
       </c>
       <c r="C381" s="4" t="inlineStr">
         <is>
-          <t>list envelopes lists are { docs: [...] }</t>
+          <t>ServiceInputSchema needs no price on request</t>
         </is>
       </c>
       <c r="D381" s="4" t="inlineStr">
@@ -10880,7 +10880,7 @@
       </c>
       <c r="C382" s="4" t="inlineStr">
         <is>
-          <t>list envelopes reference year is checked against the current year at parse time</t>
+          <t>AdminListQuerySchema caps pageSize at 100</t>
         </is>
       </c>
       <c r="D382" s="4" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="C383" s="4" t="inlineStr">
         <is>
-          <t>address only the postcode is required; blank street and city become null</t>
+          <t>parse helpers parseBody answers 400 with the issues</t>
         </is>
       </c>
       <c r="D383" s="4" t="inlineStr">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="C384" s="4" t="inlineStr">
         <is>
-          <t>service input as the app sends it a category alone is valid (the server fills currency and title)</t>
+          <t>parse helpers parseQuery reads the search params</t>
         </is>
       </c>
       <c r="D384" s="4" t="inlineStr">
@@ -10951,7 +10951,7 @@
     <row r="385">
       <c r="A385" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B385" s="4" t="inlineStr">
@@ -10961,7 +10961,7 @@
       </c>
       <c r="C385" s="4" t="inlineStr">
         <is>
-          <t>catalogue de and en have the same keys</t>
+          <t>list envelopes lists are { docs: [...] }</t>
         </is>
       </c>
       <c r="D385" s="4" t="inlineStr">
@@ -10978,7 +10978,7 @@
     <row r="386">
       <c r="A386" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B386" s="4" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="C386" s="4" t="inlineStr">
         <is>
-          <t>catalogue no text is empty and no two keys of one namespace carry the same text</t>
+          <t>list envelopes reference year is checked against the current year at parse time</t>
         </is>
       </c>
       <c r="D386" s="4" t="inlineStr">
@@ -11005,7 +11005,7 @@
     <row r="387">
       <c r="A387" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B387" s="4" t="inlineStr">
@@ -11015,7 +11015,7 @@
       </c>
       <c r="C387" s="4" t="inlineStr">
         <is>
-          <t>catalogue no text contains Treuhand, Escrow, garantiert or a competitor name</t>
+          <t>address only the postcode is required; blank street and city become null</t>
         </is>
       </c>
       <c r="D387" s="4" t="inlineStr">
@@ -11032,7 +11032,7 @@
     <row r="388">
       <c r="A388" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B388" s="4" t="inlineStr">
@@ -11042,7 +11042,7 @@
       </c>
       <c r="C388" s="4" t="inlineStr">
         <is>
-          <t>catalogue the product name is only written in brand.name</t>
+          <t>service input as the app sends it a category alone is valid (the server fills currency and title)</t>
         </is>
       </c>
       <c r="D388" s="4" t="inlineStr">
@@ -11069,7 +11069,7 @@
       </c>
       <c r="C389" s="4" t="inlineStr">
         <is>
-          <t>t replaces placeholders and falls back to the key when missing</t>
+          <t>catalogue de and en have the same keys</t>
         </is>
       </c>
       <c r="D389" s="4" t="inlineStr">
@@ -11096,7 +11096,7 @@
       </c>
       <c r="C390" s="4" t="inlineStr">
         <is>
-          <t>t fills the brand name without a parameter</t>
+          <t>catalogue no text is empty and no two keys of one namespace carry the same text</t>
         </is>
       </c>
       <c r="D390" s="4" t="inlineStr">
@@ -11123,7 +11123,7 @@
       </c>
       <c r="C391" s="4" t="inlineStr">
         <is>
-          <t>t knows its languages</t>
+          <t>catalogue no text contains Treuhand, Escrow, garantiert or a competitor name</t>
         </is>
       </c>
       <c r="D391" s="4" t="inlineStr">
@@ -11150,7 +11150,7 @@
       </c>
       <c r="C392" s="4" t="inlineStr">
         <is>
-          <t>money formats per language</t>
+          <t>catalogue the product name is only written in brand.name</t>
         </is>
       </c>
       <c r="D392" s="4" t="inlineStr">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="C393" s="4" t="inlineStr">
         <is>
-          <t>money formats price labels from the catalogue</t>
+          <t>t replaces placeholders and falls back to the key when missing</t>
         </is>
       </c>
       <c r="D393" s="4" t="inlineStr">
@@ -11204,7 +11204,7 @@
       </c>
       <c r="C394" s="4" t="inlineStr">
         <is>
-          <t>acceptLang en-GB,en;q=0.9,de;q=0.8 -&gt; en</t>
+          <t>t fills the brand name without a parameter</t>
         </is>
       </c>
       <c r="D394" s="4" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="C395" s="4" t="inlineStr">
         <is>
-          <t>acceptLang * -&gt; undefined</t>
+          <t>t knows its languages</t>
         </is>
       </c>
       <c r="D395" s="4" t="inlineStr">
@@ -11258,7 +11258,7 @@
       </c>
       <c r="C396" s="4" t="inlineStr">
         <is>
-          <t>acceptLang fr-FR -&gt; undefined</t>
+          <t>money formats per language</t>
         </is>
       </c>
       <c r="D396" s="4" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="C397" s="4" t="inlineStr">
         <is>
-          <t>acceptLang  -&gt; undefined</t>
+          <t>money formats price labels from the catalogue</t>
         </is>
       </c>
       <c r="D397" s="4" t="inlineStr">
@@ -11312,15 +11312,123 @@
       </c>
       <c r="C398" s="4" t="inlineStr">
         <is>
+          <t>acceptLang en-GB,en;q=0.9,de;q=0.8 -&gt; en</t>
+        </is>
+      </c>
+      <c r="D398" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E398" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B399" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C399" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang * -&gt; undefined</t>
+        </is>
+      </c>
+      <c r="D399" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E399" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B400" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C400" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang fr-FR -&gt; undefined</t>
+        </is>
+      </c>
+      <c r="D400" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E400" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B401" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C401" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang  -&gt; undefined</t>
+        </is>
+      </c>
+      <c r="D401" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E401" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B402" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C402" s="4" t="inlineStr">
+        <is>
           <t>acceptLang undefined -&gt; undefined</t>
         </is>
       </c>
-      <c r="D398" s="4" t="inlineStr">
+      <c r="D402" s="4" t="inlineStr">
         <is>
           <t>Packages</t>
         </is>
       </c>
-      <c r="E398" s="4" t="inlineStr">
+      <c r="E402" s="4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -11486,7 +11594,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>23 suites.</t>
+          <t>24 suites.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -11496,7 +11604,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>115 tests.</t>
+          <t>119 tests.</t>
         </is>
       </c>
     </row>
@@ -12146,7 +12254,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Creates the draft, reloads /me, then navigates; failure does not navigate; double tap runs once; welcome passes through.</t>
+          <t>Creates the draft, reloads /me, then hands the target to the tabs layout, which navigates once the tab is visible; failure sets no target; double tap runs once; welcome passes through; sign-out clears the target.</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -12156,7 +12264,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>apps/mobile start-offering.test.ts.</t>
+          <t>apps/mobile start-offering.test.ts; pending-navigation.test.ts. The layout effect itself needs a phone.</t>
         </is>
       </c>
     </row>
@@ -13103,7 +13211,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Both create the draft, reload /me and open the profile page directly (they used to fall back to Home because the tab was hidden). The sign-up tick uses the same helper. Provider card moved under the find-help button, hidden for providers. Phone checks: Offer services opens the profile page directly; the card is under the find-help button and opens the same page; a provider no longer sees the card.</t>
+          <t>Both create the draft, reload /me and open the profile page directly (they used to fall back to Home because the tab was hidden). The sign-up tick uses the same helper. Provider card moved under the find-help button, hidden for providers. Phone checks: Offer services opens the profile page directly; the card is under the find-help button and opens the same page; a provider no longer sees the card. The navigation waits for the tabs layout to show the tab (hand-off through a pending target), not for luck.</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: report and README counts after the PR review fixes
</commit_message>
<xml_diff>
--- a/Reports/Registration-Setup-Test-Report.xlsx
+++ b/Reports/Registration-Setup-Test-Report.xlsx
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Test Results'!C2:C402)</f>
+        <f>COUNTA('Test Results'!C2:C408)</f>
         <v/>
       </c>
     </row>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Results'!E2:E402,"Passed")</f>
+        <f>COUNTIF('Test Results'!E2:E408,"Passed")</f>
         <v/>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Results'!E2:E402,"Failed")</f>
+        <f>COUNTIF('Test Results'!E2:E408,"Failed")</f>
         <v/>
       </c>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Test Results'!E2:E402,"Skipped")</f>
+        <f>COUNTIF('Test Results'!E2:E408,"Skipped")</f>
         <v/>
       </c>
     </row>
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7738,17 +7738,17 @@
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>Share profile</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>share-profile.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>the provider page url carries the language only when it is not the default</t>
+          <t>set, consume once, then nothing</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
@@ -7765,17 +7765,17 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>Share profile</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>share-profile.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>shareProfile passes the url and the text in the given language</t>
+          <t>clearPending drops it (sign-out)</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
@@ -7792,17 +7792,17 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>creates the draft, reloads /me, then sets the target, in that order</t>
+          <t>readyToNavigate: only with a target and a visible profile tab</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
@@ -7819,17 +7819,17 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Pending navigation</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>pending-navigation.test.ts</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>welcome passes through</t>
+          <t>the layout order: not ready keeps the target, ready consumes it once</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
@@ -7846,17 +7846,17 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Share profile</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>share-profile.test.ts</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>a failure returns the error text and does not navigate</t>
+          <t>the provider page url carries the language only when it is not the default</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
@@ -7873,17 +7873,17 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>Start offering</t>
+          <t>Share profile</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>start-offering.test.ts</t>
+          <t>share-profile.test.ts</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>a second call while one runs does nothing extra</t>
+          <t>shareProfile passes the url and the text in the given language</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
@@ -7900,17 +7900,17 @@
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
         <is>
-          <t>Address fields</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>address-fields.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>toAddress: empty is null (clears), a postcode alone is enough, street or city without postcode is undefined</t>
+          <t>creates the draft, reloads /me, then sets the target, in that order</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr">
@@ -7927,17 +7927,17 @@
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>signUp posts email, password and name and stores the session cookie</t>
+          <t>welcome passes through</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
@@ -7954,17 +7954,17 @@
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>signIn posts email and password and returns the user</t>
+          <t>a failure returns the error text and does not navigate</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
@@ -7981,17 +7981,17 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>a refused sign-in throws the server code, which maps to a catalogue message</t>
+          <t>a second call while one runs does nothing extra</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
@@ -8008,17 +8008,17 @@
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
-          <t>signOut forgets the session at once and tells the server with the old cookie</t>
+          <t>no target when /me says the person is not a provider</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
@@ -8035,17 +8035,17 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Start offering</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>start-offering.test.ts</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr">
         <is>
-          <t>signOut offline still signs out</t>
+          <t>a sign-out during the run leaves no target behind</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
@@ -8062,17 +8062,17 @@
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Address fields</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>address-fields.test.ts</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
-          <t>session reads get-session with the cookie; no cookie means null without a request</t>
+          <t>toAddress: empty is null (clears), a postcode alone is enough, street or city without postcode is undefined</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
@@ -8094,12 +8094,12 @@
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
-          <t>session throws on a network error (the app offers a retry, not the login)</t>
+          <t>server errors land on the right field</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
@@ -8121,12 +8121,12 @@
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>sendVerificationCode asks for an email-verification code</t>
+          <t>withItem adds a trimmed new skill or strength once and ignores blanks</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
@@ -8148,12 +8148,12 @@
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>verifyEmail sends the code as otp, stores the new session and returns the user</t>
+          <t>the form-level error shows unless every server error has an inline slot</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
@@ -8175,12 +8175,12 @@
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>requestPasswordReset asks for a reset code</t>
+          <t>service and reference validation</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
@@ -8202,12 +8202,12 @@
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>resetPassword sends email, code and the new password</t>
+          <t>every missing item the publish route can return has de and en text</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
@@ -8229,12 +8229,12 @@
       </c>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>a wrong code throws INVALID_OTP, shown as the code message</t>
+          <t>the service body names the category by id and the currency, as the server expects</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
@@ -8256,12 +8256,12 @@
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>auth.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>signUp and signIn start without an old stored session</t>
+          <t>a 400 "Invalid input" marks each named field</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
@@ -8278,17 +8278,17 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>Pending navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>pending-navigation.test.ts</t>
+          <t>profile-form.test.ts</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>set, consume once, then nothing</t>
+          <t>live means published and not suspended now (the server rule of listServices)</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
@@ -8305,17 +8305,17 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>Pending navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>pending-navigation.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>clearPending drops it (sign-out)</t>
+          <t>preparePhoto keeps the long side at 1600 px</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
@@ -8332,17 +8332,17 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>Pending navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>pending-navigation.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>readyToNavigate: only with a target and a visible profile tab</t>
+          <t>tooLarge is true above 4_434_464 bytes</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
@@ -8364,12 +8364,12 @@
       </c>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>server errors land on the right field</t>
+          <t>pickPhoto cancelled is null</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
@@ -8391,12 +8391,12 @@
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>withItem adds a trimmed new skill or strength once and ignores blanks</t>
+          <t>pickPhoto a refused permission is denied, not cancelled</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
@@ -8418,12 +8418,12 @@
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>the form-level error shows unless every server error has an inline slot</t>
+          <t>pickDocument offers PDFs and the image types the server accepts, from any file source</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
@@ -8445,12 +8445,12 @@
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>pick.test.ts</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>service and reference validation</t>
+          <t>pickDocument cancelled is null</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
@@ -8472,12 +8472,12 @@
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>every missing item the publish route can return has de and en text</t>
+          <t>prices follow the website rules in German and English</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
@@ -8499,12 +8499,12 @@
       </c>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>the service body names the category by id and the currency, as the server expects</t>
+          <t>distance shows km, remote or nothing</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
@@ -8526,12 +8526,12 @@
       </c>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>a 400 "Invalid input" marks each named field</t>
+          <t>search path leaves out empty filters and trims text</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
@@ -8553,12 +8553,12 @@
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>profile-form.test.ts</t>
+          <t>format.test.ts</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>live means published and not suspended now (the server rule of listServices)</t>
+          <t>photoSrc loads only absolute http(s) URLs, never a server-relative /api path</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
@@ -8580,12 +8580,12 @@
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>preparePhoto keeps the long side at 1600 px</t>
+          <t>loading -&gt; signed in -&gt; signed out</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
@@ -8607,12 +8607,12 @@
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>tooLarge is true above 4_434_464 bytes</t>
+          <t>an unverified email never counts as signed in: sign-in sends a code and asks for it</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
@@ -8634,12 +8634,12 @@
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>pickPhoto cancelled is null</t>
+          <t>a server that refuses unverified sign-ins (EMAIL_NOT_VERIFIED) also leads to the code screen</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
@@ -8661,12 +8661,12 @@
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>pickPhoto a refused permission is denied, not cancelled</t>
+          <t>sign-up creates the account and sends the code; the right code signs in and saves the account name</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
@@ -8688,12 +8688,12 @@
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>pickDocument offers PDFs and the image types the server accepts, from any file source</t>
+          <t>a wrong code throws and keeps signed out</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
@@ -8715,12 +8715,12 @@
       </c>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>pick.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>pickDocument cancelled is null</t>
+          <t>a failed login rejects and keeps signed out; a server error on load means signed out</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
@@ -8742,12 +8742,12 @@
       </c>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>no rows when no service needs a document</t>
+          <t>a network error on load sets offline (not signed out); retry recovers</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
@@ -8769,12 +8769,12 @@
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>a babysitting service with nothing uploaded â†’ police-certificate none</t>
+          <t>onUnauthorized from the API client signs the user out</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
@@ -8796,12 +8796,12 @@
       </c>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>the most recently reviewed check decides, like the server</t>
+          <t>switching the language also saves it for emails, but only while signed in</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
@@ -8823,12 +8823,12 @@
       </c>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>a pending check shows pending even after an approval</t>
+          <t>verify finishes the sign-up: names and address, then the picture, then the record is cleared; returns the tick</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
@@ -8850,12 +8850,12 @@
       </c>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>a requirement code the app does not know still gets a row, after the known ones</t>
+          <t>a failed upload keeps the record; loadSession retries it once and clears it</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
@@ -8877,12 +8877,12 @@
       </c>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>two services needing the same document give one row</t>
+          <t>loadSession without a record or while signed out does not finish a sign-up</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
@@ -8904,12 +8904,12 @@
       </c>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>two different categories needing the same document give one row with the latest status</t>
+          <t>a record for another email is dropped and applies nothing</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
@@ -8931,12 +8931,12 @@
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>a hidden service says a document is needed until it is uploaded, then that it waits for the check</t>
+          <t>a failed PATCH keeps the full record</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
@@ -8958,12 +8958,12 @@
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>sharing is allowed only while no service waits for a document</t>
+          <t>a postcode the server calls invalid does not block the names: they are saved without the address</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
@@ -8985,12 +8985,12 @@
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>documents.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>saving a waiting service keeps Share hidden: the server answer carries waitingFor</t>
+          <t>after the PATCH succeeded, a failed upload keeps only email, tick and picture; the retry does not PATCH again</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
@@ -9007,17 +9007,17 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>Use flash</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>use-flash.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>createFlash: on after show, off after the delay, off at once on hide, a second show restarts the delay</t>
+          <t>a picture whose cached file is gone is dropped and the record cleared</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
@@ -9034,17 +9034,17 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>Use flash</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>use-flash.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>createFlash: show is a no-op after dispose</t>
+          <t>sign-up keeps the record for the code step; a failed sign-up leaves none</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
@@ -9066,12 +9066,12 @@
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>use-session.test.ts</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>prices follow the website rules in German and English</t>
+          <t>finishing a sign-up reloads /me so the home nudge sees the new picture; nothing to finish, nothing to reload</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
@@ -9093,12 +9093,12 @@
       </c>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>distance shows km, remote or nothing</t>
+          <t>signUp posts email, password and name and stores the session cookie</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
@@ -9120,12 +9120,12 @@
       </c>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>search path leaves out empty filters and trims text</t>
+          <t>signIn posts email and password and returns the user</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
@@ -9147,12 +9147,12 @@
       </c>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>format.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>photoSrc loads only absolute http(s) URLs, never a server-relative /api path</t>
+          <t>a refused sign-in throws the server code, which maps to a catalogue message</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
@@ -9174,12 +9174,12 @@
       </c>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>translation.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>applyTexts swaps only the translatable fields and keeps names, prices and photos</t>
+          <t>signOut forgets the session at once and tells the server with the old cookie</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
@@ -9201,12 +9201,12 @@
       </c>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>translation.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>applyTexts matches services and references by id and leaves unknown ones untouched</t>
+          <t>signOut offline still signs out</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
@@ -9228,12 +9228,12 @@
       </c>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>translation.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>applyTexts keeps line breaks</t>
+          <t>session reads get-session with the cookie; no cookie means null without a request</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
@@ -9255,12 +9255,12 @@
       </c>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>sends the stored cookie and stores a new set-cookie</t>
+          <t>session throws on a network error (the app offers a retry, not the login)</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
@@ -9282,12 +9282,12 @@
       </c>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>a single joined set-cookie header (no getSetCookie) is split into its cookies</t>
+          <t>sendVerificationCode asks for an email-verification code</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
@@ -9309,12 +9309,12 @@
       </c>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>clears the session on 401</t>
+          <t>verifyEmail sends the code as otp, stores the new session and returns the user</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
@@ -9336,12 +9336,12 @@
       </c>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>a 401 without a stored session does not call onUnauthorized</t>
+          <t>requestPasswordReset asks for a reset code</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
@@ -9363,12 +9363,12 @@
       </c>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>every request names the app origin and leaves the platform cookie store out</t>
+          <t>resetPassword sends email, code and the new password</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
@@ -9390,12 +9390,12 @@
       </c>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>a 409 with error and missing throws ApiError with code and missing</t>
+          <t>a wrong code throws INVALID_OTP, shown as the code message</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
@@ -9417,12 +9417,12 @@
       </c>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>auth.test.ts</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>a 400 "Invalid input" lists the fields named by its issues</t>
+          <t>signUp and signIn start without an old stored session</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
@@ -9444,12 +9444,12 @@
       </c>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>translation.test.ts</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>a network failure throws ApiError(0, network)</t>
+          <t>applyTexts swaps only the translatable fields and keeps names, prices and photos</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
@@ -9471,12 +9471,12 @@
       </c>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>translation.test.ts</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>a server that never answers fails as network after the time limit</t>
+          <t>applyTexts matches services and references by id and leaves unknown ones untouched</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
@@ -9498,12 +9498,12 @@
       </c>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>translation.test.ts</t>
         </is>
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>saves have no time limit: a slow save that succeeds is not reported as a failure</t>
+          <t>applyTexts keeps line breaks</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
@@ -9525,12 +9525,12 @@
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>my-profile.test.ts</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>updateMe PATCHes the account name</t>
+          <t>a failed check after the upload deletes the uploaded file and reports the original error</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
@@ -9552,12 +9552,12 @@
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>my-profile.test.ts</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>upload sends multipart with the cookie and no time limit</t>
+          <t>a successful submit deletes nothing</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
@@ -9579,12 +9579,12 @@
       </c>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>my-profile.test.ts</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>upload sends the file bytes with its name and type, not a bare { uri } object</t>
+          <t>a failing clean-up does not hide the original error</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
@@ -9601,17 +9601,17 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Pending signup</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>pending-signup.test.ts</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>a file the phone cannot open is "File unreadable", not a network error, and nothing is sent</t>
+          <t>the pending record round-trips and clears</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
@@ -9628,17 +9628,17 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Serial create</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>serial-create.test.ts</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>upload maps a 413 to ApiError "File too large"</t>
+          <t>choosing twice before the create returns creates once, then updates</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
@@ -9655,17 +9655,17 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Serial create</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>serial-create.test.ts</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>upload maps a network failure to ApiError network and does not retry</t>
+          <t>an existing id is only updated</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
@@ -9682,17 +9682,17 @@
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>a store that cannot be read (Keystore failure) sends the request without a cookie</t>
+          <t>two quick changes become one request with the last value</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
@@ -9709,17 +9709,17 @@
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B339" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C339" s="4" t="inlineStr">
         <is>
-          <t>a cookie that cannot be saved does not fail a request the server already carried out</t>
+          <t>flush saves immediately and nothing is sent twice</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
@@ -9736,17 +9736,17 @@
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>a malformed Set-Cookie line without "=" is skipped</t>
+          <t>a rejected save marks error and retry resends the same value</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
@@ -9763,17 +9763,17 @@
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B341" s="4" t="inlineStr">
         <is>
-          <t>client.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>updateMe sends the one-field name as first and last name, split at the last space</t>
+          <t>a change typed while a save is in flight is sent after it, in order</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -9790,17 +9790,17 @@
     <row r="342">
       <c r="A342" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use field save</t>
         </is>
       </c>
       <c r="B342" s="4" t="inlineStr">
         <is>
-          <t>my-profile.test.ts</t>
+          <t>use-field-save.test.ts</t>
         </is>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>a failed check after the upload deletes the uploaded file and reports the original error</t>
+          <t>dispose sends a pending change so nothing typed is lost</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
@@ -9822,12 +9822,12 @@
       </c>
       <c r="B343" s="4" t="inlineStr">
         <is>
-          <t>my-profile.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>a successful submit deletes nothing</t>
+          <t>sends the stored cookie and stores a new set-cookie</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
@@ -9849,12 +9849,12 @@
       </c>
       <c r="B344" s="4" t="inlineStr">
         <is>
-          <t>my-profile.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
-          <t>a failing clean-up does not hide the original error</t>
+          <t>a single joined set-cookie header (no getSetCookie) is split into its cookies</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
@@ -9871,17 +9871,17 @@
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B345" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t>two quick changes become one request with the last value</t>
+          <t>clears the session on 401</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
@@ -9898,17 +9898,17 @@
     <row r="346">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B346" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
-          <t>flush saves immediately and nothing is sent twice</t>
+          <t>a 401 without a stored session does not call onUnauthorized</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
@@ -9925,17 +9925,17 @@
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B347" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
-          <t>a rejected save marks error and retry resends the same value</t>
+          <t>every request names the app origin and leaves the platform cookie store out</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
@@ -9952,17 +9952,17 @@
     <row r="348">
       <c r="A348" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B348" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C348" s="4" t="inlineStr">
         <is>
-          <t>a change typed while a save is in flight is sent after it, in order</t>
+          <t>a 409 with error and missing throws ApiError with code and missing</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
@@ -9979,17 +9979,17 @@
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>Use field save</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B349" s="4" t="inlineStr">
         <is>
-          <t>use-field-save.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C349" s="4" t="inlineStr">
         <is>
-          <t>dispose sends a pending change so nothing typed is lost</t>
+          <t>a 400 "Invalid input" lists the fields named by its issues</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
@@ -10006,17 +10006,17 @@
     <row r="350">
       <c r="A350" s="4" t="inlineStr">
         <is>
-          <t>Stale guard</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B350" s="4" t="inlineStr">
         <is>
-          <t>stale-guard.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C350" s="4" t="inlineStr">
         <is>
-          <t>a response older than one already applied is ignored</t>
+          <t>a network failure throws ApiError(0, network)</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr">
@@ -10033,17 +10033,17 @@
     <row r="351">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t>Stale guard</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B351" s="4" t="inlineStr">
         <is>
-          <t>stale-guard.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C351" s="4" t="inlineStr">
         <is>
-          <t>answers arriving in order are all applied</t>
+          <t>a server that never answers fails as network after the time limit</t>
         </is>
       </c>
       <c r="D351" s="4" t="inlineStr">
@@ -10065,12 +10065,12 @@
       </c>
       <c r="B352" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C352" s="4" t="inlineStr">
         <is>
-          <t>loading -&gt; signed in -&gt; signed out</t>
+          <t>saves have no time limit: a slow save that succeeds is not reported as a failure</t>
         </is>
       </c>
       <c r="D352" s="4" t="inlineStr">
@@ -10092,12 +10092,12 @@
       </c>
       <c r="B353" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C353" s="4" t="inlineStr">
         <is>
-          <t>an unverified email never counts as signed in: sign-in sends a code and asks for it</t>
+          <t>updateMe PATCHes the account name</t>
         </is>
       </c>
       <c r="D353" s="4" t="inlineStr">
@@ -10119,12 +10119,12 @@
       </c>
       <c r="B354" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C354" s="4" t="inlineStr">
         <is>
-          <t>a server that refuses unverified sign-ins (EMAIL_NOT_VERIFIED) also leads to the code screen</t>
+          <t>upload sends multipart with the cookie and no time limit</t>
         </is>
       </c>
       <c r="D354" s="4" t="inlineStr">
@@ -10146,12 +10146,12 @@
       </c>
       <c r="B355" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>sign-up creates the account and sends the code; the right code signs in and saves the account name</t>
+          <t>upload sends the file bytes with its name and type, not a bare { uri } object</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr">
@@ -10173,12 +10173,12 @@
       </c>
       <c r="B356" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C356" s="4" t="inlineStr">
         <is>
-          <t>a wrong code throws and keeps signed out</t>
+          <t>a file the phone cannot open is "File unreadable", not a network error, and nothing is sent</t>
         </is>
       </c>
       <c r="D356" s="4" t="inlineStr">
@@ -10200,12 +10200,12 @@
       </c>
       <c r="B357" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C357" s="4" t="inlineStr">
         <is>
-          <t>a failed login rejects and keeps signed out; a server error on load means signed out</t>
+          <t>upload maps a 413 to ApiError "File too large"</t>
         </is>
       </c>
       <c r="D357" s="4" t="inlineStr">
@@ -10227,12 +10227,12 @@
       </c>
       <c r="B358" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C358" s="4" t="inlineStr">
         <is>
-          <t>a network error on load sets offline (not signed out); retry recovers</t>
+          <t>upload maps a network failure to ApiError network and does not retry</t>
         </is>
       </c>
       <c r="D358" s="4" t="inlineStr">
@@ -10254,12 +10254,12 @@
       </c>
       <c r="B359" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
-          <t>onUnauthorized from the API client signs the user out</t>
+          <t>a store that cannot be read (Keystore failure) sends the request without a cookie</t>
         </is>
       </c>
       <c r="D359" s="4" t="inlineStr">
@@ -10281,12 +10281,12 @@
       </c>
       <c r="B360" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C360" s="4" t="inlineStr">
         <is>
-          <t>switching the language also saves it for emails, but only while signed in</t>
+          <t>a cookie that cannot be saved does not fail a request the server already carried out</t>
         </is>
       </c>
       <c r="D360" s="4" t="inlineStr">
@@ -10308,12 +10308,12 @@
       </c>
       <c r="B361" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C361" s="4" t="inlineStr">
         <is>
-          <t>verify finishes the sign-up: names and address, then the picture, then the record is cleared; returns the tick</t>
+          <t>a malformed Set-Cookie line without "=" is skipped</t>
         </is>
       </c>
       <c r="D361" s="4" t="inlineStr">
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B362" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>client.test.ts</t>
         </is>
       </c>
       <c r="C362" s="4" t="inlineStr">
         <is>
-          <t>a failed upload keeps the record; loadSession retries it once and clears it</t>
+          <t>updateMe sends the one-field name as first and last name, split at the last space</t>
         </is>
       </c>
       <c r="D362" s="4" t="inlineStr">
@@ -10357,17 +10357,17 @@
     <row r="363">
       <c r="A363" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use me</t>
         </is>
       </c>
       <c r="B363" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-me.test.ts</t>
         </is>
       </c>
       <c r="C363" s="4" t="inlineStr">
         <is>
-          <t>loadSession without a record or while signed out does not finish a sign-up</t>
+          <t>a loadMe in flight at sign-out never fills the store for the next account</t>
         </is>
       </c>
       <c r="D363" s="4" t="inlineStr">
@@ -10384,17 +10384,17 @@
     <row r="364">
       <c r="A364" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use me</t>
         </is>
       </c>
       <c r="B364" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-me.test.ts</t>
         </is>
       </c>
       <c r="C364" s="4" t="inlineStr">
         <is>
-          <t>a record for another email is dropped and applies nothing</t>
+          <t>the newest loadMe wins: an older, slower response never overwrites a newer one</t>
         </is>
       </c>
       <c r="D364" s="4" t="inlineStr">
@@ -10411,17 +10411,17 @@
     <row r="365">
       <c r="A365" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use flash</t>
         </is>
       </c>
       <c r="B365" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-flash.test.ts</t>
         </is>
       </c>
       <c r="C365" s="4" t="inlineStr">
         <is>
-          <t>a failed PATCH keeps the full record</t>
+          <t>createFlash: on after show, off after the delay, off at once on hide, a second show restarts the delay</t>
         </is>
       </c>
       <c r="D365" s="4" t="inlineStr">
@@ -10438,17 +10438,17 @@
     <row r="366">
       <c r="A366" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use flash</t>
         </is>
       </c>
       <c r="B366" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-flash.test.ts</t>
         </is>
       </c>
       <c r="C366" s="4" t="inlineStr">
         <is>
-          <t>after the PATCH succeeded, a failed upload keeps only email, tick and picture; the retry does not PATCH again</t>
+          <t>createFlash: show is a no-op after dispose</t>
         </is>
       </c>
       <c r="D366" s="4" t="inlineStr">
@@ -10465,17 +10465,17 @@
     <row r="367">
       <c r="A367" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Use flash</t>
         </is>
       </c>
       <c r="B367" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>use-flash.test.ts</t>
         </is>
       </c>
       <c r="C367" s="4" t="inlineStr">
         <is>
-          <t>a picture whose cached file is gone is dropped and the record cleared</t>
+          <t>createFlash: a fresh flash after a dispose works again (remount)</t>
         </is>
       </c>
       <c r="D367" s="4" t="inlineStr">
@@ -10497,12 +10497,12 @@
       </c>
       <c r="B368" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>match.test.ts</t>
         </is>
       </c>
       <c r="C368" s="4" t="inlineStr">
         <is>
-          <t>sign-up keeps the record for the code step; a failed sign-up leaves none</t>
+          <t>matches ignores case and accents, and an empty query matches everything</t>
         </is>
       </c>
       <c r="D368" s="4" t="inlineStr">
@@ -10519,17 +10519,17 @@
     <row r="369">
       <c r="A369" s="4" t="inlineStr">
         <is>
-          <t>Phone app</t>
+          <t>Stale guard</t>
         </is>
       </c>
       <c r="B369" s="4" t="inlineStr">
         <is>
-          <t>use-session.test.ts</t>
+          <t>stale-guard.test.ts</t>
         </is>
       </c>
       <c r="C369" s="4" t="inlineStr">
         <is>
-          <t>finishing a sign-up reloads /me so the home nudge sees the new picture; nothing to finish, nothing to reload</t>
+          <t>a response older than one already applied is ignored</t>
         </is>
       </c>
       <c r="D369" s="4" t="inlineStr">
@@ -10546,17 +10546,17 @@
     <row r="370">
       <c r="A370" s="4" t="inlineStr">
         <is>
-          <t>Pending signup</t>
+          <t>Stale guard</t>
         </is>
       </c>
       <c r="B370" s="4" t="inlineStr">
         <is>
-          <t>pending-signup.test.ts</t>
+          <t>stale-guard.test.ts</t>
         </is>
       </c>
       <c r="C370" s="4" t="inlineStr">
         <is>
-          <t>the pending record round-trips and clears</t>
+          <t>answers arriving in order are all applied</t>
         </is>
       </c>
       <c r="D370" s="4" t="inlineStr">
@@ -10573,17 +10573,17 @@
     <row r="371">
       <c r="A371" s="4" t="inlineStr">
         <is>
-          <t>Picture nudge</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B371" s="4" t="inlineStr">
         <is>
-          <t>picture-nudge.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C371" s="4" t="inlineStr">
         <is>
-          <t>the dismissed-nudge key is per user, so a second account on the device still sees it</t>
+          <t>no rows when no service needs a document</t>
         </is>
       </c>
       <c r="D371" s="4" t="inlineStr">
@@ -10605,12 +10605,12 @@
       </c>
       <c r="B372" s="4" t="inlineStr">
         <is>
-          <t>match.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C372" s="4" t="inlineStr">
         <is>
-          <t>matches ignores case and accents, and an empty query matches everything</t>
+          <t>a babysitting service with nothing uploaded â†’ police-certificate none</t>
         </is>
       </c>
       <c r="D372" s="4" t="inlineStr">
@@ -10627,17 +10627,17 @@
     <row r="373">
       <c r="A373" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B373" s="4" t="inlineStr">
         <is>
-          <t>profile-tab.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C373" s="4" t="inlineStr">
         <is>
-          <t>the My profile tab shows only for a known provider</t>
+          <t>the most recently reviewed check decides, like the server</t>
         </is>
       </c>
       <c r="D373" s="4" t="inlineStr">
@@ -10654,17 +10654,17 @@
     <row r="374">
       <c r="A374" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B374" s="4" t="inlineStr">
         <is>
-          <t>profile-tab.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C374" s="4" t="inlineStr">
         <is>
-          <t>after sign-out the next account does not inherit the provider tab</t>
+          <t>a pending check shows pending even after an approval</t>
         </is>
       </c>
       <c r="D374" s="4" t="inlineStr">
@@ -10686,12 +10686,12 @@
       </c>
       <c r="B375" s="4" t="inlineStr">
         <is>
-          <t>auth-layout.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C375" s="4" t="inlineStr">
         <is>
-          <t>logged-out landing route is login</t>
+          <t>a requirement code the app does not know still gets a row, after the known ones</t>
         </is>
       </c>
       <c r="D375" s="4" t="inlineStr">
@@ -10713,12 +10713,12 @@
       </c>
       <c r="B376" s="4" t="inlineStr">
         <is>
-          <t>auth-layout.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C376" s="4" t="inlineStr">
         <is>
-          <t>no test files inside src/app (each file there becomes a screen)</t>
+          <t>two services needing the same document give one row</t>
         </is>
       </c>
       <c r="D376" s="4" t="inlineStr">
@@ -10735,17 +10735,17 @@
     <row r="377">
       <c r="A377" s="4" t="inlineStr">
         <is>
-          <t>Serial create</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B377" s="4" t="inlineStr">
         <is>
-          <t>serial-create.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C377" s="4" t="inlineStr">
         <is>
-          <t>choosing twice before the create returns creates once, then updates</t>
+          <t>two different categories needing the same document give one row with the latest status</t>
         </is>
       </c>
       <c r="D377" s="4" t="inlineStr">
@@ -10762,17 +10762,17 @@
     <row r="378">
       <c r="A378" s="4" t="inlineStr">
         <is>
-          <t>Serial create</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B378" s="4" t="inlineStr">
         <is>
-          <t>serial-create.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C378" s="4" t="inlineStr">
         <is>
-          <t>an existing id is only updated</t>
+          <t>a hidden service says a document is needed until it is uploaded, then that it waits for the check</t>
         </is>
       </c>
       <c r="D378" s="4" t="inlineStr">
@@ -10789,17 +10789,17 @@
     <row r="379">
       <c r="A379" s="4" t="inlineStr">
         <is>
-          <t>Use me</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B379" s="4" t="inlineStr">
         <is>
-          <t>use-me.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C379" s="4" t="inlineStr">
         <is>
-          <t>a loadMe in flight at sign-out never fills the store for the next account</t>
+          <t>sharing is allowed only while no service waits for a document</t>
         </is>
       </c>
       <c r="D379" s="4" t="inlineStr">
@@ -10816,22 +10816,22 @@
     <row r="380">
       <c r="A380" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B380" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>documents.test.ts</t>
         </is>
       </c>
       <c r="C380" s="4" t="inlineStr">
         <is>
-          <t>ServiceInputSchema rejects three decimals and negative prices</t>
+          <t>saving a waiting service keeps Share hidden: the server answer carries waitingFor</t>
         </is>
       </c>
       <c r="D380" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E380" s="4" t="inlineStr">
@@ -10843,22 +10843,22 @@
     <row r="381">
       <c r="A381" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B381" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>profile-tab.test.ts</t>
         </is>
       </c>
       <c r="C381" s="4" t="inlineStr">
         <is>
-          <t>ServiceInputSchema needs no price on request</t>
+          <t>the My profile tab shows only for a known provider</t>
         </is>
       </c>
       <c r="D381" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E381" s="4" t="inlineStr">
@@ -10870,22 +10870,22 @@
     <row r="382">
       <c r="A382" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B382" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>profile-tab.test.ts</t>
         </is>
       </c>
       <c r="C382" s="4" t="inlineStr">
         <is>
-          <t>AdminListQuerySchema caps pageSize at 100</t>
+          <t>after sign-out the next account does not inherit the provider tab</t>
         </is>
       </c>
       <c r="D382" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E382" s="4" t="inlineStr">
@@ -10897,22 +10897,22 @@
     <row r="383">
       <c r="A383" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Picture nudge</t>
         </is>
       </c>
       <c r="B383" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>picture-nudge.test.ts</t>
         </is>
       </c>
       <c r="C383" s="4" t="inlineStr">
         <is>
-          <t>parse helpers parseBody answers 400 with the issues</t>
+          <t>the dismissed-nudge key is per user, so a second account on the device still sees it</t>
         </is>
       </c>
       <c r="D383" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E383" s="4" t="inlineStr">
@@ -10924,22 +10924,22 @@
     <row r="384">
       <c r="A384" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B384" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>auth-layout.test.ts</t>
         </is>
       </c>
       <c r="C384" s="4" t="inlineStr">
         <is>
-          <t>parse helpers parseQuery reads the search params</t>
+          <t>logged-out landing route is login</t>
         </is>
       </c>
       <c r="D384" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E384" s="4" t="inlineStr">
@@ -10951,22 +10951,22 @@
     <row r="385">
       <c r="A385" s="4" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>Phone app</t>
         </is>
       </c>
       <c r="B385" s="4" t="inlineStr">
         <is>
-          <t>index.test.ts</t>
+          <t>auth-layout.test.ts</t>
         </is>
       </c>
       <c r="C385" s="4" t="inlineStr">
         <is>
-          <t>list envelopes lists are { docs: [...] }</t>
+          <t>no test files inside src/app (each file there becomes a screen)</t>
         </is>
       </c>
       <c r="D385" s="4" t="inlineStr">
         <is>
-          <t>Packages</t>
+          <t>App</t>
         </is>
       </c>
       <c r="E385" s="4" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="C386" s="4" t="inlineStr">
         <is>
-          <t>list envelopes reference year is checked against the current year at parse time</t>
+          <t>ServiceInputSchema rejects three decimals and negative prices</t>
         </is>
       </c>
       <c r="D386" s="4" t="inlineStr">
@@ -11015,7 +11015,7 @@
       </c>
       <c r="C387" s="4" t="inlineStr">
         <is>
-          <t>address only the postcode is required; blank street and city become null</t>
+          <t>ServiceInputSchema needs no price on request</t>
         </is>
       </c>
       <c r="D387" s="4" t="inlineStr">
@@ -11042,7 +11042,7 @@
       </c>
       <c r="C388" s="4" t="inlineStr">
         <is>
-          <t>service input as the app sends it a category alone is valid (the server fills currency and title)</t>
+          <t>AdminListQuerySchema caps pageSize at 100</t>
         </is>
       </c>
       <c r="D388" s="4" t="inlineStr">
@@ -11059,7 +11059,7 @@
     <row r="389">
       <c r="A389" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B389" s="4" t="inlineStr">
@@ -11069,7 +11069,7 @@
       </c>
       <c r="C389" s="4" t="inlineStr">
         <is>
-          <t>catalogue de and en have the same keys</t>
+          <t>parse helpers parseBody answers 400 with the issues</t>
         </is>
       </c>
       <c r="D389" s="4" t="inlineStr">
@@ -11086,7 +11086,7 @@
     <row r="390">
       <c r="A390" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B390" s="4" t="inlineStr">
@@ -11096,7 +11096,7 @@
       </c>
       <c r="C390" s="4" t="inlineStr">
         <is>
-          <t>catalogue no text is empty and no two keys of one namespace carry the same text</t>
+          <t>parse helpers parseQuery reads the search params</t>
         </is>
       </c>
       <c r="D390" s="4" t="inlineStr">
@@ -11113,7 +11113,7 @@
     <row r="391">
       <c r="A391" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B391" s="4" t="inlineStr">
@@ -11123,7 +11123,7 @@
       </c>
       <c r="C391" s="4" t="inlineStr">
         <is>
-          <t>catalogue no text contains Treuhand, Escrow, garantiert or a competitor name</t>
+          <t>list envelopes lists are { docs: [...] }</t>
         </is>
       </c>
       <c r="D391" s="4" t="inlineStr">
@@ -11140,7 +11140,7 @@
     <row r="392">
       <c r="A392" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B392" s="4" t="inlineStr">
@@ -11150,7 +11150,7 @@
       </c>
       <c r="C392" s="4" t="inlineStr">
         <is>
-          <t>catalogue the product name is only written in brand.name</t>
+          <t>list envelopes reference year is checked against the current year at parse time</t>
         </is>
       </c>
       <c r="D392" s="4" t="inlineStr">
@@ -11167,7 +11167,7 @@
     <row r="393">
       <c r="A393" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B393" s="4" t="inlineStr">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="C393" s="4" t="inlineStr">
         <is>
-          <t>t replaces placeholders and falls back to the key when missing</t>
+          <t>address only the postcode is required; blank street and city become null</t>
         </is>
       </c>
       <c r="D393" s="4" t="inlineStr">
@@ -11194,7 +11194,7 @@
     <row r="394">
       <c r="A394" s="4" t="inlineStr">
         <is>
-          <t>Texts</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="B394" s="4" t="inlineStr">
@@ -11204,7 +11204,7 @@
       </c>
       <c r="C394" s="4" t="inlineStr">
         <is>
-          <t>t fills the brand name without a parameter</t>
+          <t>service input as the app sends it a category alone is valid (the server fills currency and title)</t>
         </is>
       </c>
       <c r="D394" s="4" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="C395" s="4" t="inlineStr">
         <is>
-          <t>t knows its languages</t>
+          <t>catalogue de and en have the same keys</t>
         </is>
       </c>
       <c r="D395" s="4" t="inlineStr">
@@ -11258,7 +11258,7 @@
       </c>
       <c r="C396" s="4" t="inlineStr">
         <is>
-          <t>money formats per language</t>
+          <t>catalogue no text is empty and no two keys of one namespace carry the same text</t>
         </is>
       </c>
       <c r="D396" s="4" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="C397" s="4" t="inlineStr">
         <is>
-          <t>money formats price labels from the catalogue</t>
+          <t>catalogue no text contains Treuhand, Escrow, garantiert or a competitor name</t>
         </is>
       </c>
       <c r="D397" s="4" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="C398" s="4" t="inlineStr">
         <is>
-          <t>acceptLang en-GB,en;q=0.9,de;q=0.8 -&gt; en</t>
+          <t>catalogue the product name is only written in brand.name</t>
         </is>
       </c>
       <c r="D398" s="4" t="inlineStr">
@@ -11339,7 +11339,7 @@
       </c>
       <c r="C399" s="4" t="inlineStr">
         <is>
-          <t>acceptLang * -&gt; undefined</t>
+          <t>t replaces placeholders and falls back to the key when missing</t>
         </is>
       </c>
       <c r="D399" s="4" t="inlineStr">
@@ -11366,7 +11366,7 @@
       </c>
       <c r="C400" s="4" t="inlineStr">
         <is>
-          <t>acceptLang fr-FR -&gt; undefined</t>
+          <t>t fills the brand name without a parameter</t>
         </is>
       </c>
       <c r="D400" s="4" t="inlineStr">
@@ -11393,7 +11393,7 @@
       </c>
       <c r="C401" s="4" t="inlineStr">
         <is>
-          <t>acceptLang  -&gt; undefined</t>
+          <t>t knows its languages</t>
         </is>
       </c>
       <c r="D401" s="4" t="inlineStr">
@@ -11420,15 +11420,177 @@
       </c>
       <c r="C402" s="4" t="inlineStr">
         <is>
+          <t>money formats per language</t>
+        </is>
+      </c>
+      <c r="D402" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E402" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B403" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C403" s="4" t="inlineStr">
+        <is>
+          <t>money formats price labels from the catalogue</t>
+        </is>
+      </c>
+      <c r="D403" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E403" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B404" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C404" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang en-GB,en;q=0.9,de;q=0.8 -&gt; en</t>
+        </is>
+      </c>
+      <c r="D404" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E404" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B405" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C405" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang * -&gt; undefined</t>
+        </is>
+      </c>
+      <c r="D405" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E405" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B406" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C406" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang fr-FR -&gt; undefined</t>
+        </is>
+      </c>
+      <c r="D406" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E406" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B407" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C407" s="4" t="inlineStr">
+        <is>
+          <t>acceptLang  -&gt; undefined</t>
+        </is>
+      </c>
+      <c r="D407" s="4" t="inlineStr">
+        <is>
+          <t>Packages</t>
+        </is>
+      </c>
+      <c r="E407" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="4" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B408" s="4" t="inlineStr">
+        <is>
+          <t>index.test.ts</t>
+        </is>
+      </c>
+      <c r="C408" s="4" t="inlineStr">
+        <is>
           <t>acceptLang undefined -&gt; undefined</t>
         </is>
       </c>
-      <c r="D402" s="4" t="inlineStr">
+      <c r="D408" s="4" t="inlineStr">
         <is>
           <t>Packages</t>
         </is>
       </c>
-      <c r="E402" s="4" t="inlineStr">
+      <c r="E408" s="4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -11604,7 +11766,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>119 tests.</t>
+          <t>125 tests.</t>
         </is>
       </c>
     </row>
@@ -12345,7 +12507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -13220,6 +13382,23 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Fixed (PR review): offering, postcode, saving</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>The newest /me request wins; Offer services needs isProvider true and leaves no target after a sign-out; the layout consumes the target only when the tab is visible; the server checks the postcode format (400 Invalid postcode; a well-formed unlisted one is accepted); a refused sign-up postcode no longer blocks the names; Account fields are locked while saving. Phone check: Offer services reaches the My profile tab route (not the empty app/my-profile stack); a bad postcode shows the new text in Account.</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Fixed; Not yet done (phone)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>